<commit_message>
docs: add broader neurotropic panel negative result to tracking workbook Notes
HIV/coronavirus(incl. SARS-CoV-2)/hepatitis A-E/poliovirus/enterovirus/
rabies/West Nile/JC polyomavirus/measles/mumps/Zika -- zero hits, all 9
cohorts, zero threshold. Real negative result, not just unchecked -- same
weight as the existing VZV/CMV/EBV finding.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/neurotrophic_virus_tracking.xlsx
+++ b/docs/neurotrophic_virus_tracking.xlsx
@@ -6061,7 +6061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -6176,7 +6176,7 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Cross-species hits not yet resolved as artifact vs. real divergent signal -- same open question as the existing Cytomegalovirus papiinebeta3 -&gt; "Human CMV proxy" precedent in assets/taxon_remap.tsv. Thoracic DRG's 80T2R carries both human HSV-1 (38 reads) AND atelinealpha1 (58 reads) in the same sample -- suggestive of divergent-read k-mer splitting. The other 3 off-species-only samples (111T9R, 114T12R, 473-1) have no co-occurring human signal -- less clear.</t>
+          <t>Broader neurotropic/systemic virus panel (zero-threshold, all 9 cohorts, terms: 'immunodeficiency virus', 'coronavir', 'hepatitis', 'poliovirus', 'enterovirus', 'rabies', 'lyssavirus', 'west nile', 'polyomavirus', 'measles', 'morbillivirus', 'mumps', 'rubulavirus', 'zika') -- completely clean, zero hits in any cohort at any read count. Covers HIV, all coronaviruses incl. SARS-CoV-2, hepatitis A-E, poliovirus/enterovirus, rabies/lyssavirus, West Nile virus, JC polyomavirus, measles/mumps, Zika. Real negative, same weight as the VZV/CMV/EBV finding above -- not just unchecked.</t>
         </is>
       </c>
     </row>
@@ -6186,31 +6186,31 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Two artifact-candidate taxa observed in Tier 1 (dual-DB) output, NOT yet broken out per-sample in the By Sample tab (only seen as cohort-level taxon-name hits so far):</t>
+          <t>Cross-species hits not yet resolved as artifact vs. real divergent signal -- same open question as the existing Cytomegalovirus papiinebeta3 -&gt; "Human CMV proxy" precedent in assets/taxon_remap.tsv. Thoracic DRG's 80T2R carries both human HSV-1 (38 reads) AND atelinealpha1 (58 reads) in the same sample -- suggestive of divergent-read k-mer splitting. The other 3 off-species-only samples (111T9R, 114T12R, 473-1) have no co-occurring human signal -- less clear.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Mus musculus mobilized endogenous polytropic provirus (590745) -- murine retrovirus, seen in BOTH Watchmaker (~7-taxon murine cluster) and dpn_ra_kulkarni (2 unrelated cohorts) -- looks like a recurring database/k-mer cross-mapping artifact, same class as the existing hantavirus/orthobunyavirus entries in assets/artifact_taxa.tsv, not yet added to that list.</t>
-        </is>
-      </c>
+      <c r="A22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Lilac leaf chlorosis virus (722755) -- plant virus, osm_juliet only so far. No biological plausibility in human tissue -- same class as existing Gihfavirus/Kinglevirus artifact entries.</t>
+          <t>Two artifact-candidate taxa observed in Tier 1 (dual-DB) output, NOT yet broken out per-sample in the By Sample tab (only seen as cohort-level taxon-name hits so far):</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr"/>
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Mus musculus mobilized endogenous polytropic provirus (590745) -- murine retrovirus, seen in BOTH Watchmaker (~7-taxon murine cluster) and dpn_ra_kulkarni (2 unrelated cohorts) -- looks like a recurring database/k-mer cross-mapping artifact, same class as the existing hantavirus/orthobunyavirus entries in assets/artifact_taxa.tsv, not yet added to that list.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>104T8R (Thoracic DRG) is a confirmed genuine library failure -- 92 total STAR input reads. Saad-2 (mgoexplant_saad) independently confirms a pre-existing "known library failure" flag via zero HERV-K even at raw threshold.</t>
+          <t xml:space="preserve">  - Lilac leaf chlorosis virus (722755) -- plant virus, osm_juliet only so far. No biological plausibility in human tissue -- same class as existing Gihfavirus/Kinglevirus artifact entries.</t>
         </is>
       </c>
     </row>
@@ -6219,6 +6219,16 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>104T8R (Thoracic DRG) is a confirmed genuine library failure -- 92 total STAR input reads. Saad-2 (mgoexplant_saad) independently confirms a pre-existing "known library failure" flag via zero HERV-K even at raw threshold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>Source: virome pipeline (github.com/mwilde49/virome-pipeline), 2026-08-19 gataca-&gt;Titan-&gt;scratch batch. Full detail: Claude memory project_neurotrophic_virus_screen_2026-08.md and project_hervk_findings.md.</t>
         </is>

</xml_diff>

<commit_message>
docs: full-inventory sweep synthesis in tracking workbook Notes
~130-taxon 'vir'-substring inventory across all 9 cohorts (bracken_raw, zero
threshold, deduplicated) -- mostly expected background matching existing
artifact_taxa.tsv categories. Two real updates: (1) the murine-retrovirus
finding is bigger than thought -- 15+ animal retrovirus/sarcoma-virus names
together, likely one HERV-K/endogenous-retroviral cross-mapping phenomenon
across the whole Retroviridae tree, not isolated contamination; (2) Molluscum
contagiosum virus is a real human poxvirus finding, not an artifact.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/neurotrophic_virus_tracking.xlsx
+++ b/docs/neurotrophic_virus_tracking.xlsx
@@ -6061,7 +6061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -6220,15 +6220,39 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>104T8R (Thoracic DRG) is a confirmed genuine library failure -- 92 total STAR input reads. Saad-2 (mgoexplant_saad) independently confirms a pre-existing "known library failure" flag via zero HERV-K even at raw threshold.</t>
+          <t>Full 'vir'-substring inventory (bracken_raw, zero threshold, all 9 cohorts, deduplicated) surfaced ~130 distinct taxa -- mostly expected viral-metagenomics background (30+ bacteriophage genera; the already-documented giant-amoeba-virus, ruminant-orthobunyavirus/ hantavirus, and avian-herpesvirus artifact categories from assets/artifact_taxa.tsv; plant/insect/fish viruses matching the existing Gihfavirus/Kinglevirus DRG environmental cross-mapping precedent). Two things worth keeping from that sweep:</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr"/>
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - The murine-retrovirus finding above is actually much bigger: 15+ distinct animal retrovirus/sarcoma-virus names together (murine, feline, avian, monkey leukemia/sarcoma viruses, plus Alpha/Beta/Gammaretrovirus genus levels). Retroviruses share deep gag/pol/env homology, so this looks like ONE underlying phenomenon -- HERV-K or other endogenous retroviral sequence cross-mapping across the whole Retroviridae tree via Kraken2 LCA -- not 15 separate contamination events.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Molluscum contagiosum virus (10279, genus Molluscipoxvirus) is a real, common human-infecting poxvirus, NOT an artifact candidate like the rest of this list -- a legitimate, if non-neurotrophic, incidental pathogen finding worth keeping in mind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>104T8R (Thoracic DRG) is a confirmed genuine library failure -- 92 total STAR input reads. Saad-2 (mgoexplant_saad) independently confirms a pre-existing "known library failure" flag via zero HERV-K even at raw threshold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>Source: virome pipeline (github.com/mwilde49/virome-pipeline), 2026-08-19 gataca-&gt;Titan-&gt;scratch batch. Full detail: Claude memory project_neurotrophic_virus_screen_2026-08.md and project_hervk_findings.md.</t>
         </is>

</xml_diff>